<commit_message>
add description to code
</commit_message>
<xml_diff>
--- a/results/res_table.xlsx
+++ b/results/res_table.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -419,42 +419,42 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2.200***</t>
+          <t>2.132***</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>(0.488)</t>
+          <t>(0.420)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2.213***</t>
+          <t>2.212***</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>(0.358)</t>
+          <t>(0.521)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2.186***</t>
+          <t>2.210***</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>(0.391)</t>
+          <t>(0.532)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2.507***</t>
+          <t>2.665***</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>(0.384)</t>
+          <t>(0.622)</t>
         </is>
       </c>
     </row>
@@ -471,42 +471,42 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.880***</t>
+          <t>1.936***</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>(0.474)</t>
+          <t>(0.504)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.892***</t>
+          <t>2.057***</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>(0.333)</t>
+          <t>(0.547)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.935***</t>
+          <t>2.045***</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>(0.285)</t>
+          <t>(0.512)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.020***</t>
+          <t>2.229***</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>(0.311)</t>
+          <t>(0.627)</t>
         </is>
       </c>
     </row>
@@ -523,42 +523,42 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>-5.991***</t>
+          <t>-2.931***</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>(0.434)</t>
+          <t>(0.214)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>-6.130***</t>
+          <t>-3.213***</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>(0.347)</t>
+          <t>(0.306)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.847***</t>
+          <t>-4.827***</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>(0.875)</t>
+          <t>(0.992)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>-6.933***</t>
+          <t>-4.860***</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>(0.781)</t>
+          <t>(0.943)</t>
         </is>
       </c>
     </row>
@@ -575,42 +575,42 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.756***</t>
+          <t>1.901***</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>(0.441)</t>
+          <t>(0.384)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3.783***</t>
+          <t>2.153***</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>(0.448)</t>
+          <t>(0.452)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3.972***</t>
+          <t>3.327***</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>(0.514)</t>
+          <t>(0.623)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.722***</t>
+          <t>2.915***</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>(0.460)</t>
+          <t>(0.573)</t>
         </is>
       </c>
     </row>
@@ -627,42 +627,42 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.253***</t>
+          <t>0.236***</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>(0.048)</t>
+          <t>(0.041)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.244***</t>
+          <t>0.234***</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>(0.057)</t>
+          <t>(0.050)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.199*</t>
+          <t>0.188**</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>(0.083)</t>
+          <t>(0.063)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.173</t>
+          <t>0.155**</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>(0.112)</t>
+          <t>(0.058)</t>
         </is>
       </c>
     </row>
@@ -674,47 +674,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>uni$uu ego</t>
+          <t>Overall maximum convergence ratio</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.214</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>(0.558)</t>
+          <t>0.165</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.172</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>(0.524)</t>
+          <t>0.179</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.103</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>(0.469)</t>
+          <t>0.272</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0.456</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>(0.440)</t>
+          <t>0.263</t>
         </is>
       </c>
     </row>
@@ -726,27 +706,37 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Overall maximum convergence ratio</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0.357</t>
+          <t>gender alter</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.263</t>
+          <t>-0.306</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>(0.289)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.281</t>
+          <t>-0.044</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>(0.297)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>0.258</t>
+          <t>-0.104</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>(0.312)</t>
         </is>
       </c>
     </row>
@@ -758,37 +748,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>gender alter</t>
+          <t>gender ego</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.229</t>
+          <t>0.973**</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>(0.427)</t>
+          <t>(0.359)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.243</t>
+          <t>0.824*</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>(0.317)</t>
+          <t>(0.398)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>-0.166</t>
+          <t>0.726*</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>(0.235)</t>
+          <t>(0.350)</t>
         </is>
       </c>
     </row>
@@ -800,37 +790,37 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>gender ego</t>
+          <t>same gender</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.888*</t>
+          <t>0.236</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>(0.445)</t>
+          <t>(0.270)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.779+</t>
+          <t>0.238</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>(0.432)</t>
+          <t>(0.286)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0.496</t>
+          <t>0.224</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>(0.349)</t>
+          <t>(0.259)</t>
         </is>
       </c>
     </row>
@@ -842,37 +832,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>same gender</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>0.282</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>(0.236)</t>
+          <t>funcs[[1]] alter</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.276</t>
+          <t>2.166*</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>(0.215)</t>
+          <t>(0.975)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.249</t>
+          <t>2.128*</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>(0.197)</t>
+          <t>(0.955)</t>
         </is>
       </c>
     </row>
@@ -884,27 +864,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>funcs[[1]] alter</t>
+          <t>funcs[[1]] ego</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1.354</t>
+          <t>-0.270</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>(0.849)</t>
+          <t>(0.424)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>0.849</t>
+          <t>-0.241</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>(0.870)</t>
+          <t>(0.457)</t>
         </is>
       </c>
     </row>
@@ -916,27 +896,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>funcs[[1]] ego</t>
+          <t>funcs[[2]] alter</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.408</t>
+          <t>2.597**</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>(1.194)</t>
+          <t>(0.992)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>-1.508*</t>
+          <t>2.377**</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>(0.725)</t>
+          <t>(0.901)</t>
         </is>
       </c>
     </row>
@@ -948,27 +928,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>funcs[[2]] alter</t>
+          <t>funcs[[2]] ego</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2.615***</t>
+          <t>-1.754**</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>(0.667)</t>
+          <t>(0.601)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.831**</t>
+          <t>-2.015***</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>(0.657)</t>
+          <t>(0.596)</t>
         </is>
       </c>
     </row>
@@ -980,27 +960,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>funcs[[2]] ego</t>
+          <t>funcs[[3]] alter</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-2.534*</t>
+          <t>2.646*</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>(1.095)</t>
+          <t>(1.148)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>-2.919***</t>
+          <t>2.553*</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>(0.803)</t>
+          <t>(1.067)</t>
         </is>
       </c>
     </row>
@@ -1012,27 +992,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>funcs[[3]] alter</t>
+          <t>funcs[[3]] ego</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2.616***</t>
+          <t>-0.833</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>(0.710)</t>
+          <t>(1.025)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1.801*</t>
+          <t>-1.129</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>(0.701)</t>
+          <t>(0.971)</t>
         </is>
       </c>
     </row>
@@ -1044,27 +1024,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>funcs[[3]] ego</t>
+          <t>funcs[[4]] alter</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-1.889+</t>
+          <t>2.515*</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>(1.075)</t>
+          <t>(1.064)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>-2.553*</t>
+          <t>2.455*</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>(0.993)</t>
+          <t>(0.960)</t>
         </is>
       </c>
     </row>
@@ -1076,27 +1056,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>funcs[[4]] alter</t>
+          <t>funcs[[4]] ego</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2.562**</t>
+          <t>-1.792*</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>(0.808)</t>
+          <t>(0.713)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1.924*</t>
+          <t>-2.039**</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>(0.870)</t>
+          <t>(0.710)</t>
         </is>
       </c>
     </row>
@@ -1108,27 +1088,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>funcs[[4]] ego</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>-0.806</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>(0.893)</t>
+          <t>dissim</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.594*</t>
+          <t>-4.032***</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>(0.718)</t>
+          <t>(1.180)</t>
         </is>
       </c>
     </row>
@@ -1140,17 +1110,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>dissim</t>
+          <t>distan</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>-3.825***</t>
+          <t>-0.201</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>(1.032)</t>
+          <t>(0.208)</t>
         </is>
       </c>
     </row>
@@ -1162,17 +1132,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>distan</t>
+          <t>intdis alter</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-2.569***</t>
+          <t>0.797</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>(0.545)</t>
+          <t>(1.261)</t>
         </is>
       </c>
     </row>
@@ -1184,39 +1154,69 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>intdis alter</t>
+          <t>intdis ego</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.083</t>
+          <t>1.021</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>(0.825)</t>
+          <t>(1.394)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>first</t>
+          <t>last</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>intdis ego</t>
+          <t>constant last rate (period 1)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3.562***</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>(0.728)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>3.579***</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>(0.924)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>5.062**</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>(1.771)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>-1.280</t>
+          <t>6.739**</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>(1.410)</t>
+          <t>(2.088)</t>
         </is>
       </c>
     </row>
@@ -1228,47 +1228,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>constant last rate (period 1)</t>
+          <t>constant last rate (period 2)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>3.701***</t>
+          <t>2.428***</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>(0.804)</t>
+          <t>(0.704)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3.725***</t>
+          <t>2.382***</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>(0.834)</t>
+          <t>(0.536)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>4.420***</t>
+          <t>2.848***</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>(0.698)</t>
+          <t>(0.830)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>4.899***</t>
+          <t>3.103***</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>(0.807)</t>
+          <t>(0.833)</t>
         </is>
       </c>
     </row>
@@ -1280,47 +1280,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>constant last rate (period 2)</t>
+          <t>outdegree (density)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2.914***</t>
+          <t>-2.309***</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(0.499)</t>
+          <t>(0.365)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2.876***</t>
+          <t>-2.414***</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>(0.388)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>-3.872***</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>(0.679)</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>3.339***</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>(0.502)</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>3.389***</t>
+          <t>-3.852***</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>(0.549)</t>
+          <t>(0.811)</t>
         </is>
       </c>
     </row>
@@ -1332,47 +1332,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>outdegree (density)</t>
+          <t>reciprocity</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>-7.086***</t>
+          <t>1.452***</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>(0.314)</t>
+          <t>(0.395)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>-7.241***</t>
+          <t>1.508***</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>(0.435)</t>
+          <t>(0.386)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>-11.357***</t>
+          <t>1.655***</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>(1.367)</t>
+          <t>(0.457)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>-10.103***</t>
+          <t>1.101*</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>(1.161)</t>
+          <t>(0.500)</t>
         </is>
       </c>
     </row>
@@ -1384,47 +1384,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>reciprocity</t>
+          <t>indegree - popularity</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3.204***</t>
+          <t>-0.045</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(0.493)</t>
+          <t>(0.152)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>3.203***</t>
+          <t>-0.046</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>(0.525)</t>
+          <t>(0.151)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2.409***</t>
+          <t>-0.124</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>(0.463)</t>
+          <t>(0.167)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1.401***</t>
+          <t>-0.393+</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>(0.407)</t>
+          <t>(0.222)</t>
         </is>
       </c>
     </row>
@@ -1436,47 +1436,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>indegree - popularity</t>
+          <t>Overall maximum convergence ratio</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.301**</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>(0.092)</t>
+          <t>0.165</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0.300+</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>(0.157)</t>
+          <t>0.179</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0.254</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>(873.527)</t>
+          <t>0.272</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>0.201*</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>(0.087)</t>
+          <t>0.263</t>
         </is>
       </c>
     </row>
@@ -1488,47 +1468,37 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>uni$uu ego</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1.928**</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>(0.653)</t>
+          <t>gender alter</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.882**</t>
+          <t>0.058</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>(0.624)</t>
+          <t>(0.257)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0.839**</t>
+          <t>0.159</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>(0.321)</t>
+          <t>(0.313)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>1.179***</t>
+          <t>-0.030</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>(0.326)</t>
+          <t>(0.316)</t>
         </is>
       </c>
     </row>
@@ -1540,27 +1510,37 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Overall maximum convergence ratio</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>0.357</t>
+          <t>gender ego</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0.263</t>
+          <t>-0.175</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>(0.348)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.281</t>
+          <t>0.473</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>(0.456)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>0.258</t>
+          <t>-0.067</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>(0.418)</t>
         </is>
       </c>
     </row>
@@ -1572,37 +1552,37 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>gender alter</t>
+          <t>same gender</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0.392</t>
+          <t>0.189</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>(0.321)</t>
+          <t>(0.227)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0.391*</t>
+          <t>0.154</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>(0.179)</t>
+          <t>(0.248)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>0.372*</t>
+          <t>0.072</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>(0.180)</t>
+          <t>(0.258)</t>
         </is>
       </c>
     </row>
@@ -1614,37 +1594,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>gender ego</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>-0.236</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>(0.387)</t>
+          <t>funcs[[1]] alter</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>-0.218</t>
+          <t>0.894*</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>(0.318)</t>
+          <t>(0.431)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>-0.288</t>
+          <t>0.868</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>(0.310)</t>
+          <t>(0.570)</t>
         </is>
       </c>
     </row>
@@ -1656,37 +1626,27 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>same gender</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>0.282</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>(0.197)</t>
+          <t>funcs[[1]] ego</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0.230</t>
+          <t>-1.056</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>(0.165)</t>
+          <t>(1.396)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>0.223</t>
+          <t>-1.053</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>(0.201)</t>
+          <t>(1.289)</t>
         </is>
       </c>
     </row>
@@ -1698,27 +1658,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>funcs[[1]] alter</t>
+          <t>funcs[[2]] alter</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0.463</t>
+          <t>0.951*</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>(0.532)</t>
+          <t>(0.373)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>-0.056</t>
+          <t>0.833+</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>(0.487)</t>
+          <t>(0.441)</t>
         </is>
       </c>
     </row>
@@ -1730,27 +1690,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>funcs[[1]] ego</t>
+          <t>funcs[[2]] ego</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2.248</t>
+          <t>0.793</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>(1.654)</t>
+          <t>(0.632)</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>1.110</t>
+          <t>0.596</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>(1.630)</t>
+          <t>(0.677)</t>
         </is>
       </c>
     </row>
@@ -1762,27 +1722,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>funcs[[2]] alter</t>
+          <t>funcs[[3]] alter</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0.723</t>
+          <t>0.886</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>(0.446)</t>
+          <t>(0.642)</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>0.022</t>
+          <t>0.939</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>(0.416)</t>
+          <t>(0.776)</t>
         </is>
       </c>
     </row>
@@ -1794,27 +1754,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>funcs[[2]] ego</t>
+          <t>funcs[[3]] ego</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>4.993**</t>
+          <t>2.356**</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>(1.601)</t>
+          <t>(0.802)</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>3.438*</t>
+          <t>1.900*</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>(1.386)</t>
+          <t>(0.811)</t>
         </is>
       </c>
     </row>
@@ -1826,27 +1786,27 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>funcs[[3]] alter</t>
+          <t>funcs[[4]] alter</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.214</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>(0.539)</t>
+          <t>(0.516)</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>-0.010</t>
+          <t>0.094</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>(0.461)</t>
+          <t>(0.552)</t>
         </is>
       </c>
     </row>
@@ -1858,27 +1818,27 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>funcs[[3]] ego</t>
+          <t>funcs[[4]] ego</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>6.598***</t>
+          <t>2.100**</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>(1.465)</t>
+          <t>(0.679)</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>4.734***</t>
+          <t>1.924*</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>(1.307)</t>
+          <t>(0.777)</t>
         </is>
       </c>
     </row>
@@ -1890,27 +1850,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>funcs[[4]] alter</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>0.590</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>(0.439)</t>
+          <t>dissim</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>-0.271</t>
+          <t>-6.270***</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>(0.466)</t>
+          <t>(1.555)</t>
         </is>
       </c>
     </row>
@@ -1922,27 +1872,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>funcs[[4]] ego</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>6.612***</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>(1.425)</t>
+          <t>distan</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>4.809***</t>
+          <t>-0.272</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>(1.382)</t>
+          <t>(0.208)</t>
         </is>
       </c>
     </row>
@@ -1954,17 +1894,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>dissim</t>
+          <t>intdis alter</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>-4.265***</t>
+          <t>1.297</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>(0.835)</t>
+          <t>(1.415)</t>
         </is>
       </c>
     </row>
@@ -1976,61 +1916,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>distan</t>
+          <t>intdis ego</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>-1.601***</t>
+          <t>-1.592</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>(0.289)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>last</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>intdis alter</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>0.645</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>(0.763)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>last</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>intdis ego</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>-0.527</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>(0.995)</t>
+          <t>(1.747)</t>
         </is>
       </c>
     </row>

</xml_diff>